<commit_message>
Updated firebase config keys
</commit_message>
<xml_diff>
--- a/temp_reg.xlsx
+++ b/temp_reg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1adbb6d4af469bba/Documents/Talawakelle Divisional Secretariat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:4000b_{06888659-485A-4030-BF3E-A45EB180120C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CC29200-A568-4E5C-A110-32B99FA09911}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:4000b_{06888659-485A-4030-BF3E-A45EB180120C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0827D741-43A7-4C67-A8E3-2C6D9678D752}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -574,7 +574,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -746,6 +746,21 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1147,7 +1162,7 @@
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="42" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1180,6 +1195,8 @@
     <xf numFmtId="0" fontId="23" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="47">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1241,6 +1258,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2617,18 +2638,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C35"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="23.4"/>
   <cols>
-    <col min="1" max="1" width="28.77734375" customWidth="1"/>
-    <col min="2" max="2" width="34.88671875" customWidth="1"/>
+    <col min="1" max="2" width="41.21875" style="13" customWidth="1"/>
     <col min="3" max="3" width="17.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="12" t="s">
         <v>82</v>
       </c>
       <c r="C1" t="s">
@@ -2636,154 +2656,154 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="A2" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="13" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="A3" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="13" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="A4" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="13" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" t="s">
+      <c r="A5" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="13" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" t="s">
+      <c r="A6" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="13" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" t="s">
+      <c r="A7" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="13" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" t="s">
+      <c r="A8" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="13" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" t="s">
+      <c r="A9" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="13" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:3">
-      <c r="A10" t="s">
+      <c r="A10" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="13" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:3">
-      <c r="A11" t="s">
+      <c r="A11" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="13" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" t="s">
+      <c r="A12" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="13" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:3">
-      <c r="A13" t="s">
+      <c r="A13" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="13" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" t="s">
+      <c r="A14" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="13" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" t="s">
+      <c r="A15" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="13" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:3">
-      <c r="A16" t="s">
+      <c r="A16" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="13" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:3">
-      <c r="A17" t="s">
+      <c r="A17" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="13" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:3">
-      <c r="A18" t="s">
+      <c r="A18" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="13" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:3">
-      <c r="A19" t="s">
+      <c r="A19" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="13" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="20" spans="1:3">
-      <c r="A20" t="s">
+      <c r="A20" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="13" t="s">
         <v>137</v>
       </c>
       <c r="C20" t="s">
@@ -2791,128 +2811,129 @@
       </c>
     </row>
     <row r="21" spans="1:3">
-      <c r="A21" t="s">
+      <c r="A21" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="13" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="22" spans="1:3">
-      <c r="A22" t="s">
+      <c r="A22" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="13" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:3">
-      <c r="A23" t="s">
+      <c r="A23" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="13" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" t="s">
+      <c r="A24" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="13" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:3">
-      <c r="A25" t="s">
+      <c r="A25" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="13" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:3">
-      <c r="A26" t="s">
+      <c r="A26" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="13" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="27" spans="1:3">
-      <c r="A27" t="s">
+      <c r="A27" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="28" spans="1:3">
-      <c r="A28" t="s">
+      <c r="A28" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="13" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:3">
-      <c r="A29" t="s">
+      <c r="A29" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="13" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="30" spans="1:3">
-      <c r="A30" t="s">
+      <c r="A30" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="13" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="31" spans="1:3">
-      <c r="A31" t="s">
+      <c r="A31" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="13" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:3">
-      <c r="A32" t="s">
+      <c r="A32" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="13" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="33" spans="1:2">
-      <c r="A33" t="s">
+      <c r="A33" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="13" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="34" spans="1:2">
-      <c r="A34" t="s">
+      <c r="A34" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="13" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="35" spans="1:2">
-      <c r="A35" t="s">
+      <c r="A35" s="13" t="s">
         <v>165</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="13" t="s">
         <v>171</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:C35" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>